<commit_message>
Chore(Config) : requirements.txt 경량화 및 개발계획서 업데이트
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/상세개발계획서 AI담당.xlsx
+++ b/docs/상세개발계획서 AI담당.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sungjonghyun/3-1/산학프로젝트/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sungjonghyun/3-1/산학프로젝트/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88467AA7-C7D4-634B-B565-FCCEAC28D635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D2C4BF4-F5DC-0844-A25A-91EC00E46BBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="61">
   <si>
     <t>Task</t>
   </si>
@@ -341,10 +341,6 @@
     <phoneticPr fontId="10" type="noConversion"/>
   </si>
   <si>
-    <t>vlm 통합 모델 고려</t>
-    <phoneticPr fontId="10" type="noConversion"/>
-  </si>
-  <si>
     <t>냉장고 전체인식
 → YOLO, vlm</t>
     <phoneticPr fontId="10" type="noConversion"/>
@@ -355,6 +351,117 @@
   </si>
   <si>
     <t>정확도에 대한 기준 데이터셋 정의 후 성능 테스트</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>VLM 하이브리드 통합 모델</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>자동라벨링(미인식 데이터 자동 라벨링 파이프라인 구축)</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>타 파트 연동 준비(백엔드 연동용 추론 결과 반환 규격)</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>AI 디렉터리 전면 개편 및 Git 연동 세팅</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>Git 연동 세팅</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>√</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>FastAPI 서버 구축</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>신뢰도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> 75%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>미만 시 VLM(Gemini) 추론 연동</t>
+    </r>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Self-improving </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>기반</t>
+    </r>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ngrok </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">외부접속 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">, bearer </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Malgun Gothic"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>토큰 인증</t>
+    </r>
     <phoneticPr fontId="10" type="noConversion"/>
   </si>
 </sst>
@@ -1264,19 +1371,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -1287,6 +1381,19 @@
       <bottom style="thin">
         <color rgb="FFFFFFFF"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -1411,10 +1518,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1423,11 +1527,74 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1440,18 +1607,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1486,6 +1641,9 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1501,59 +1659,8 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1775,7 +1882,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z996"/>
+  <dimension ref="A1:AA999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.1640625" customWidth="1"/>
@@ -1786,13 +1893,13 @@
     <col min="6" max="6" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="12" width="5.83203125" bestFit="1" customWidth="1"/>
     <col min="13" max="19" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="17.5" customWidth="1"/>
+    <col min="20" max="20" width="40.1640625" customWidth="1"/>
     <col min="21" max="22" width="5.1640625" customWidth="1"/>
     <col min="23" max="23" width="9.33203125" customWidth="1"/>
     <col min="24" max="26" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="16.5" customHeight="1">
+    <row r="1" spans="1:27" ht="16.5" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1820,28 +1927,28 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="42.75" customHeight="1">
+    <row r="2" spans="1:27" ht="42.75" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-      <c r="E2" s="70"/>
-      <c r="F2" s="70"/>
-      <c r="G2" s="70"/>
-      <c r="H2" s="70"/>
-      <c r="I2" s="70"/>
-      <c r="J2" s="70"/>
-      <c r="K2" s="70"/>
-      <c r="L2" s="70"/>
-      <c r="M2" s="70"/>
-      <c r="N2" s="70"/>
-      <c r="O2" s="70"/>
-      <c r="P2" s="70"/>
-      <c r="Q2" s="70"/>
-      <c r="R2" s="70"/>
-      <c r="S2" s="49"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
+      <c r="Q2" s="43"/>
+      <c r="R2" s="43"/>
+      <c r="S2" s="44"/>
       <c r="T2" s="1"/>
       <c r="U2" s="1"/>
       <c r="V2" s="1"/>
@@ -1850,26 +1957,26 @@
       <c r="Y2" s="1"/>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:26" ht="42.75" customHeight="1">
+    <row r="3" spans="1:27" ht="42.75" customHeight="1">
       <c r="A3" s="1"/>
-      <c r="B3" s="51"/>
-      <c r="C3" s="71"/>
-      <c r="D3" s="71"/>
-      <c r="E3" s="71"/>
-      <c r="F3" s="71"/>
-      <c r="G3" s="71"/>
-      <c r="H3" s="71"/>
-      <c r="I3" s="71"/>
-      <c r="J3" s="71"/>
-      <c r="K3" s="71"/>
-      <c r="L3" s="71"/>
-      <c r="M3" s="71"/>
-      <c r="N3" s="71"/>
-      <c r="O3" s="71"/>
-      <c r="P3" s="71"/>
-      <c r="Q3" s="71"/>
-      <c r="R3" s="71"/>
-      <c r="S3" s="52"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
+      <c r="I3" s="46"/>
+      <c r="J3" s="46"/>
+      <c r="K3" s="46"/>
+      <c r="L3" s="46"/>
+      <c r="M3" s="46"/>
+      <c r="N3" s="46"/>
+      <c r="O3" s="46"/>
+      <c r="P3" s="46"/>
+      <c r="Q3" s="46"/>
+      <c r="R3" s="46"/>
+      <c r="S3" s="47"/>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
@@ -1878,26 +1985,26 @@
       <c r="Y3" s="1"/>
       <c r="Z3" s="1"/>
     </row>
-    <row r="4" spans="1:26" ht="16.5" customHeight="1" thickBot="1">
+    <row r="4" spans="1:27" ht="16.5" customHeight="1" thickBot="1">
       <c r="A4" s="1"/>
-      <c r="B4" s="72"/>
-      <c r="C4" s="73"/>
-      <c r="D4" s="73"/>
-      <c r="E4" s="73"/>
-      <c r="F4" s="73"/>
-      <c r="G4" s="73"/>
-      <c r="H4" s="73"/>
-      <c r="I4" s="73"/>
-      <c r="J4" s="73"/>
-      <c r="K4" s="73"/>
-      <c r="L4" s="73"/>
-      <c r="M4" s="73"/>
-      <c r="N4" s="73"/>
-      <c r="O4" s="73"/>
-      <c r="P4" s="73"/>
-      <c r="Q4" s="73"/>
-      <c r="R4" s="73"/>
-      <c r="S4" s="73"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="49"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="49"/>
+      <c r="K4" s="49"/>
+      <c r="L4" s="49"/>
+      <c r="M4" s="49"/>
+      <c r="N4" s="49"/>
+      <c r="O4" s="49"/>
+      <c r="P4" s="49"/>
+      <c r="Q4" s="49"/>
+      <c r="R4" s="49"/>
+      <c r="S4" s="49"/>
       <c r="T4" s="1"/>
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
@@ -1906,16 +2013,16 @@
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
     </row>
-    <row r="5" spans="1:26" ht="29.25" customHeight="1">
+    <row r="5" spans="1:27" ht="29.25" customHeight="1">
       <c r="A5" s="1"/>
-      <c r="B5" s="74" t="s">
+      <c r="B5" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="49"/>
-      <c r="D5" s="75" t="s">
+      <c r="C5" s="44"/>
+      <c r="D5" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="78" t="s">
+      <c r="E5" s="56" t="s">
         <v>2</v>
       </c>
       <c r="F5" s="2" t="s">
@@ -1924,25 +2031,25 @@
       <c r="G5" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="66" t="s">
+      <c r="H5" s="83" t="s">
         <v>5</v>
       </c>
-      <c r="I5" s="67"/>
-      <c r="J5" s="67"/>
-      <c r="K5" s="67"/>
-      <c r="L5" s="68"/>
-      <c r="M5" s="81" t="s">
+      <c r="I5" s="84"/>
+      <c r="J5" s="84"/>
+      <c r="K5" s="84"/>
+      <c r="L5" s="85"/>
+      <c r="M5" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="N5" s="84"/>
-      <c r="O5" s="84"/>
-      <c r="P5" s="85"/>
-      <c r="Q5" s="81" t="s">
+      <c r="N5" s="62"/>
+      <c r="O5" s="62"/>
+      <c r="P5" s="63"/>
+      <c r="Q5" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="R5" s="82"/>
-      <c r="S5" s="83"/>
-      <c r="T5" s="43" t="s">
+      <c r="R5" s="60"/>
+      <c r="S5" s="61"/>
+      <c r="T5" s="64" t="s">
         <v>8</v>
       </c>
       <c r="U5" s="1"/>
@@ -1952,12 +2059,12 @@
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
     </row>
-    <row r="6" spans="1:26" ht="29.25" customHeight="1">
+    <row r="6" spans="1:27" ht="29.25" customHeight="1">
       <c r="A6" s="1"/>
-      <c r="B6" s="50"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="76"/>
-      <c r="E6" s="79"/>
+      <c r="B6" s="51"/>
+      <c r="C6" s="52"/>
+      <c r="D6" s="54"/>
+      <c r="E6" s="57"/>
       <c r="F6" s="3" t="s">
         <v>9</v>
       </c>
@@ -2000,23 +2107,25 @@
       <c r="S6" s="27">
         <v>17</v>
       </c>
-      <c r="T6" s="44"/>
+      <c r="T6" s="52"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="W6" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="V6" s="1"/>
+      <c r="W6" s="1"/>
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
-    </row>
-    <row r="7" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+      <c r="Z6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="AA6" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" ht="29.25" customHeight="1" thickBot="1">
       <c r="A7" s="1"/>
-      <c r="B7" s="51"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="77"/>
-      <c r="E7" s="80"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="55"/>
+      <c r="E7" s="58"/>
       <c r="F7" s="7" t="s">
         <v>12</v>
       </c>
@@ -2059,29 +2168,31 @@
       <c r="S7" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="T7" s="44"/>
+      <c r="T7" s="52"/>
       <c r="U7" s="1"/>
-      <c r="V7" s="6"/>
-      <c r="W7" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="1"/>
-    </row>
-    <row r="8" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+      <c r="Z7" s="6"/>
+      <c r="AA7" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" ht="29.25" customHeight="1" thickBot="1">
       <c r="A8" s="1"/>
-      <c r="B8" s="48" t="s">
+      <c r="B8" s="68" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="49"/>
+      <c r="C8" s="44"/>
       <c r="D8" s="9" t="s">
         <v>43</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="63"/>
-      <c r="G8" s="56"/>
+      <c r="F8" s="79"/>
+      <c r="G8" s="72"/>
       <c r="H8" s="36" t="s">
         <v>10</v>
       </c>
@@ -2090,14 +2201,14 @@
       <c r="K8" s="20"/>
       <c r="L8" s="19"/>
       <c r="M8" s="19"/>
-      <c r="N8" s="64" t="s">
+      <c r="N8" s="81" t="s">
         <v>27</v>
       </c>
       <c r="O8" s="21"/>
       <c r="P8" s="21"/>
       <c r="Q8" s="21"/>
       <c r="R8" s="21"/>
-      <c r="S8" s="45" t="s">
+      <c r="S8" s="65" t="s">
         <v>28</v>
       </c>
       <c r="T8" s="11"/>
@@ -2107,18 +2218,18 @@
       <c r="X8" s="1"/>
       <c r="Y8" s="1"/>
     </row>
-    <row r="9" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="9" spans="1:27" ht="29.25" customHeight="1" thickBot="1">
       <c r="A9" s="1"/>
-      <c r="B9" s="50"/>
-      <c r="C9" s="44"/>
+      <c r="B9" s="51"/>
+      <c r="C9" s="52"/>
       <c r="D9" s="12" t="s">
         <v>33</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F9" s="60"/>
-      <c r="G9" s="57"/>
+      <c r="F9" s="76"/>
+      <c r="G9" s="73"/>
       <c r="H9" s="36" t="s">
         <v>10</v>
       </c>
@@ -2127,12 +2238,12 @@
       <c r="K9" s="20"/>
       <c r="L9" s="19"/>
       <c r="M9" s="19"/>
-      <c r="N9" s="46"/>
+      <c r="N9" s="66"/>
       <c r="O9" s="19"/>
       <c r="P9" s="19"/>
       <c r="Q9" s="19"/>
       <c r="R9" s="19"/>
-      <c r="S9" s="46"/>
+      <c r="S9" s="66"/>
       <c r="T9" s="11"/>
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
@@ -2140,18 +2251,18 @@
       <c r="X9" s="1"/>
       <c r="Y9" s="1"/>
     </row>
-    <row r="10" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="10" spans="1:27" ht="29.25" customHeight="1" thickBot="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="50"/>
-      <c r="C10" s="44"/>
+      <c r="B10" s="51"/>
+      <c r="C10" s="52"/>
       <c r="D10" s="12" t="s">
         <v>44</v>
       </c>
       <c r="E10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="60"/>
-      <c r="G10" s="57"/>
+      <c r="F10" s="76"/>
+      <c r="G10" s="73"/>
       <c r="H10" s="36" t="s">
         <v>10</v>
       </c>
@@ -2162,111 +2273,122 @@
       <c r="K10" s="20"/>
       <c r="L10" s="19"/>
       <c r="M10" s="19"/>
-      <c r="N10" s="46"/>
+      <c r="N10" s="66"/>
       <c r="O10" s="19"/>
       <c r="P10" s="19"/>
       <c r="Q10" s="19"/>
       <c r="R10" s="19"/>
-      <c r="S10" s="46"/>
-      <c r="T10" s="11"/>
-      <c r="U10" s="1"/>
+      <c r="S10" s="66"/>
+      <c r="T10" s="1"/>
       <c r="V10" s="1"/>
       <c r="W10" s="1"/>
       <c r="X10" s="1"/>
       <c r="Y10" s="1"/>
     </row>
-    <row r="11" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="11" spans="1:27" ht="29.25" customHeight="1" thickBot="1">
       <c r="A11" s="1"/>
-      <c r="B11" s="50"/>
-      <c r="C11" s="44"/>
+      <c r="B11" s="51"/>
+      <c r="C11" s="52"/>
       <c r="D11" s="12" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="60"/>
-      <c r="G11" s="57"/>
+      <c r="F11" s="76"/>
+      <c r="G11" s="73"/>
       <c r="H11" s="19"/>
       <c r="I11" s="19"/>
       <c r="J11" s="19"/>
-      <c r="K11" s="41"/>
-      <c r="L11" s="41"/>
+      <c r="K11" s="40"/>
+      <c r="L11" s="6" t="s">
+        <v>10</v>
+      </c>
       <c r="M11" s="19"/>
-      <c r="N11" s="46"/>
+      <c r="N11" s="66"/>
       <c r="O11" s="19"/>
       <c r="P11" s="19"/>
       <c r="Q11" s="19"/>
       <c r="R11" s="19"/>
-      <c r="S11" s="46"/>
-      <c r="T11" s="11"/>
+      <c r="S11" s="66"/>
+      <c r="T11" s="41" t="s">
+        <v>58</v>
+      </c>
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
       <c r="X11" s="1"/>
       <c r="Y11" s="1"/>
     </row>
-    <row r="12" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="12" spans="1:27" ht="29.25" customHeight="1" thickBot="1">
       <c r="A12" s="1"/>
-      <c r="B12" s="79"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="13" t="s">
-        <v>34</v>
+      <c r="B12" s="57"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="86" t="s">
+        <v>52</v>
       </c>
       <c r="E12" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="86"/>
-      <c r="G12" s="57"/>
+      <c r="F12" s="80"/>
+      <c r="G12" s="73"/>
       <c r="H12" s="19"/>
-      <c r="I12" s="36" t="s">
+      <c r="I12" s="21"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="J12" s="36" t="s">
-        <v>10</v>
-      </c>
-      <c r="K12" s="36" t="s">
-        <v>10</v>
-      </c>
-      <c r="L12" s="19"/>
       <c r="M12" s="19"/>
-      <c r="N12" s="46"/>
+      <c r="N12" s="66"/>
       <c r="O12" s="19"/>
       <c r="P12" s="19"/>
       <c r="Q12" s="19"/>
       <c r="R12" s="19"/>
-      <c r="S12" s="46"/>
-      <c r="T12" s="11"/>
+      <c r="S12" s="66"/>
+      <c r="T12" s="11" t="s">
+        <v>59</v>
+      </c>
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
       <c r="W12" s="1"/>
       <c r="X12" s="1"/>
       <c r="Y12" s="1"/>
     </row>
-    <row r="13" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="13" spans="1:27" ht="29.25" customHeight="1" thickBot="1">
       <c r="A13" s="1"/>
-      <c r="B13" s="51"/>
+      <c r="B13" s="57"/>
       <c r="C13" s="52"/>
       <c r="D13" s="13" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F13" s="61"/>
-      <c r="G13" s="58"/>
+      <c r="F13" s="80"/>
+      <c r="G13" s="73"/>
       <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="19"/>
-      <c r="K13" s="19"/>
-      <c r="L13" s="19"/>
-      <c r="M13" s="19"/>
-      <c r="N13" s="46"/>
+      <c r="I13" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="J13" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="K13" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M13" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="N13" s="66"/>
       <c r="O13" s="19"/>
       <c r="P13" s="19"/>
       <c r="Q13" s="19"/>
       <c r="R13" s="19"/>
-      <c r="S13" s="46"/>
+      <c r="S13" s="66"/>
       <c r="T13" s="11"/>
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
@@ -2274,34 +2396,32 @@
       <c r="X13" s="1"/>
       <c r="Y13" s="1"/>
     </row>
-    <row r="14" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="14" spans="1:27" ht="29.25" customHeight="1" thickBot="1">
       <c r="A14" s="1"/>
-      <c r="B14" s="53" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="49"/>
-      <c r="D14" s="9" t="s">
-        <v>42</v>
+      <c r="B14" s="57"/>
+      <c r="C14" s="52"/>
+      <c r="D14" s="13" t="s">
+        <v>53</v>
       </c>
       <c r="E14" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F14" s="63"/>
-      <c r="G14" s="56"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="36" t="s">
+      <c r="F14" s="80"/>
+      <c r="G14" s="73"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
+      <c r="L14" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="J14" s="21"/>
-      <c r="K14" s="22"/>
-      <c r="L14" s="21"/>
-      <c r="M14" s="21"/>
-      <c r="N14" s="46"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="66"/>
       <c r="O14" s="19"/>
       <c r="P14" s="19"/>
       <c r="Q14" s="19"/>
       <c r="R14" s="19"/>
-      <c r="S14" s="46"/>
+      <c r="S14" s="66"/>
       <c r="T14" s="11"/>
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
@@ -2309,32 +2429,34 @@
       <c r="X14" s="1"/>
       <c r="Y14" s="1"/>
     </row>
-    <row r="15" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="15" spans="1:27" ht="29.25" customHeight="1" thickBot="1">
       <c r="A15" s="1"/>
-      <c r="B15" s="50"/>
-      <c r="C15" s="44"/>
-      <c r="D15" s="9" t="s">
-        <v>35</v>
+      <c r="B15" s="57"/>
+      <c r="C15" s="52"/>
+      <c r="D15" s="13" t="s">
+        <v>54</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F15" s="60"/>
-      <c r="G15" s="57"/>
+      <c r="F15" s="80"/>
+      <c r="G15" s="73"/>
       <c r="H15" s="19"/>
-      <c r="I15" s="41"/>
-      <c r="J15" s="36" t="s">
+      <c r="I15" s="19"/>
+      <c r="J15" s="19"/>
+      <c r="K15" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="K15" s="20"/>
-      <c r="L15" s="19"/>
+      <c r="L15" s="36" t="s">
+        <v>10</v>
+      </c>
       <c r="M15" s="19"/>
-      <c r="N15" s="46"/>
+      <c r="N15" s="66"/>
       <c r="O15" s="19"/>
       <c r="P15" s="19"/>
       <c r="Q15" s="19"/>
       <c r="R15" s="19"/>
-      <c r="S15" s="46"/>
+      <c r="S15" s="66"/>
       <c r="T15" s="11"/>
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
@@ -2342,32 +2464,30 @@
       <c r="X15" s="1"/>
       <c r="Y15" s="1"/>
     </row>
-    <row r="16" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="16" spans="1:27" ht="29.25" customHeight="1" thickBot="1">
       <c r="A16" s="1"/>
-      <c r="B16" s="50"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="12" t="s">
-        <v>41</v>
+      <c r="B16" s="45"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="13" t="s">
+        <v>50</v>
       </c>
       <c r="E16" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F16" s="60"/>
-      <c r="G16" s="57"/>
+      <c r="F16" s="77"/>
+      <c r="G16" s="74"/>
       <c r="H16" s="19"/>
-      <c r="I16" s="40"/>
-      <c r="J16" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="K16" s="20"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
       <c r="L16" s="19"/>
       <c r="M16" s="19"/>
-      <c r="N16" s="46"/>
+      <c r="N16" s="66"/>
       <c r="O16" s="19"/>
       <c r="P16" s="19"/>
       <c r="Q16" s="19"/>
       <c r="R16" s="19"/>
-      <c r="S16" s="46"/>
+      <c r="S16" s="66"/>
       <c r="T16" s="11"/>
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
@@ -2375,30 +2495,34 @@
       <c r="X16" s="1"/>
       <c r="Y16" s="1"/>
     </row>
-    <row r="17" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="17" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A17" s="1"/>
-      <c r="B17" s="50"/>
+      <c r="B17" s="69" t="s">
+        <v>32</v>
+      </c>
       <c r="C17" s="44"/>
-      <c r="D17" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" s="10"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="57"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="6" t="s">
+      <c r="D17" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F17" s="79"/>
+      <c r="G17" s="72"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="K17" s="20"/>
-      <c r="L17" s="19"/>
-      <c r="M17" s="19"/>
-      <c r="N17" s="46"/>
+      <c r="J17" s="21"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="21"/>
+      <c r="M17" s="21"/>
+      <c r="N17" s="66"/>
       <c r="O17" s="19"/>
       <c r="P17" s="19"/>
       <c r="Q17" s="19"/>
       <c r="R17" s="19"/>
-      <c r="S17" s="46"/>
+      <c r="S17" s="66"/>
       <c r="T17" s="11"/>
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
@@ -2406,26 +2530,32 @@
       <c r="X17" s="1"/>
       <c r="Y17" s="1"/>
     </row>
-    <row r="18" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="18" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A18" s="1"/>
       <c r="B18" s="51"/>
       <c r="C18" s="52"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="61"/>
-      <c r="G18" s="58"/>
+      <c r="D18" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="76"/>
+      <c r="G18" s="73"/>
       <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="36" t="s">
+        <v>10</v>
+      </c>
       <c r="K18" s="20"/>
       <c r="L18" s="19"/>
       <c r="M18" s="19"/>
-      <c r="N18" s="46"/>
+      <c r="N18" s="66"/>
       <c r="O18" s="19"/>
       <c r="P18" s="19"/>
       <c r="Q18" s="19"/>
       <c r="R18" s="19"/>
-      <c r="S18" s="46"/>
+      <c r="S18" s="66"/>
       <c r="T18" s="11"/>
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
@@ -2433,66 +2563,65 @@
       <c r="X18" s="1"/>
       <c r="Y18" s="1"/>
     </row>
-    <row r="19" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="19" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A19" s="1"/>
-      <c r="B19" s="54" t="s">
-        <v>49</v>
-      </c>
-      <c r="C19" s="49"/>
-      <c r="D19" s="14" t="s">
-        <v>39</v>
+      <c r="B19" s="51"/>
+      <c r="C19" s="52"/>
+      <c r="D19" s="12" t="s">
+        <v>41</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F19" s="59"/>
-      <c r="G19" s="62"/>
+      <c r="F19" s="76"/>
+      <c r="G19" s="73"/>
       <c r="H19" s="19"/>
-      <c r="I19" s="36" t="s">
+      <c r="I19" s="39"/>
+      <c r="J19" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="J19" s="19"/>
       <c r="K19" s="20"/>
       <c r="L19" s="19"/>
       <c r="M19" s="19"/>
-      <c r="N19" s="46"/>
+      <c r="N19" s="66"/>
       <c r="O19" s="19"/>
       <c r="P19" s="19"/>
       <c r="Q19" s="19"/>
       <c r="R19" s="19"/>
-      <c r="S19" s="46"/>
-      <c r="T19" s="42" t="s">
-        <v>47</v>
-      </c>
+      <c r="S19" s="66"/>
+      <c r="T19" s="11"/>
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
       <c r="W19" s="1"/>
       <c r="X19" s="1"/>
       <c r="Y19" s="1"/>
     </row>
-    <row r="20" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="20" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A20" s="1"/>
-      <c r="B20" s="50"/>
-      <c r="C20" s="44"/>
+      <c r="B20" s="51"/>
+      <c r="C20" s="52"/>
       <c r="D20" s="12" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E20" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F20" s="60"/>
-      <c r="G20" s="57"/>
+      <c r="F20" s="76"/>
+      <c r="G20" s="73"/>
       <c r="H20" s="19"/>
       <c r="I20" s="19"/>
+      <c r="J20" s="6" t="s">
+        <v>10</v>
+      </c>
       <c r="K20" s="20"/>
       <c r="L20" s="19"/>
       <c r="M20" s="19"/>
-      <c r="N20" s="46"/>
+      <c r="N20" s="66"/>
       <c r="O20" s="19"/>
       <c r="P20" s="19"/>
       <c r="Q20" s="19"/>
       <c r="R20" s="19"/>
-      <c r="S20" s="46"/>
+      <c r="S20" s="66"/>
       <c r="T20" s="11"/>
       <c r="U20" s="1"/>
       <c r="V20" s="1"/>
@@ -2500,26 +2629,32 @@
       <c r="X20" s="1"/>
       <c r="Y20" s="1"/>
     </row>
-    <row r="21" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="21" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A21" s="1"/>
-      <c r="B21" s="50"/>
-      <c r="C21" s="44"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="60"/>
-      <c r="G21" s="57"/>
+      <c r="B21" s="45"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F21" s="77"/>
+      <c r="G21" s="74"/>
       <c r="H21" s="19"/>
       <c r="I21" s="19"/>
       <c r="J21" s="19"/>
       <c r="K21" s="20"/>
       <c r="L21" s="19"/>
-      <c r="M21" s="19"/>
-      <c r="N21" s="46"/>
+      <c r="M21" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="N21" s="66"/>
       <c r="O21" s="19"/>
       <c r="P21" s="19"/>
       <c r="Q21" s="19"/>
       <c r="R21" s="19"/>
-      <c r="S21" s="46"/>
+      <c r="S21" s="66"/>
       <c r="T21" s="11"/>
       <c r="U21" s="1"/>
       <c r="V21" s="1"/>
@@ -2527,55 +2662,66 @@
       <c r="X21" s="1"/>
       <c r="Y21" s="1"/>
     </row>
-    <row r="22" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="22" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A22" s="1"/>
-      <c r="B22" s="50"/>
+      <c r="B22" s="70" t="s">
+        <v>48</v>
+      </c>
       <c r="C22" s="44"/>
-      <c r="D22" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="E22" s="10"/>
-      <c r="F22" s="60"/>
-      <c r="G22" s="57"/>
+      <c r="D22" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F22" s="75"/>
+      <c r="G22" s="78"/>
       <c r="H22" s="19"/>
-      <c r="I22" s="19"/>
+      <c r="I22" s="36" t="s">
+        <v>10</v>
+      </c>
       <c r="J22" s="19"/>
-      <c r="K22" s="19"/>
-      <c r="L22" s="40"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="19"/>
       <c r="M22" s="19"/>
-      <c r="N22" s="46"/>
+      <c r="N22" s="66"/>
       <c r="O22" s="19"/>
       <c r="P22" s="19"/>
       <c r="Q22" s="19"/>
       <c r="R22" s="19"/>
-      <c r="S22" s="46"/>
-      <c r="T22" s="11"/>
+      <c r="S22" s="66"/>
+      <c r="T22" s="41" t="s">
+        <v>47</v>
+      </c>
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
       <c r="W22" s="1"/>
       <c r="X22" s="1"/>
       <c r="Y22" s="1"/>
     </row>
-    <row r="23" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="23" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A23" s="1"/>
-      <c r="B23" s="50"/>
-      <c r="C23" s="44"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="60"/>
-      <c r="G23" s="57"/>
+      <c r="B23" s="51"/>
+      <c r="C23" s="52"/>
+      <c r="D23" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F23" s="76"/>
+      <c r="G23" s="73"/>
       <c r="H23" s="19"/>
       <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
       <c r="K23" s="20"/>
       <c r="L23" s="19"/>
       <c r="M23" s="19"/>
-      <c r="N23" s="46"/>
+      <c r="N23" s="66"/>
       <c r="O23" s="19"/>
       <c r="P23" s="19"/>
       <c r="Q23" s="19"/>
       <c r="R23" s="19"/>
-      <c r="S23" s="46"/>
+      <c r="S23" s="66"/>
       <c r="T23" s="11"/>
       <c r="U23" s="1"/>
       <c r="V23" s="1"/>
@@ -2583,25 +2729,26 @@
       <c r="X23" s="1"/>
       <c r="Y23" s="1"/>
     </row>
-    <row r="24" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="24" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A24" s="1"/>
       <c r="B24" s="51"/>
       <c r="C24" s="52"/>
-      <c r="D24" s="13"/>
+      <c r="D24" s="12"/>
       <c r="E24" s="10"/>
-      <c r="F24" s="61"/>
-      <c r="G24" s="58"/>
+      <c r="F24" s="76"/>
+      <c r="G24" s="73"/>
       <c r="H24" s="19"/>
       <c r="I24" s="19"/>
+      <c r="J24" s="19"/>
       <c r="K24" s="20"/>
       <c r="L24" s="19"/>
       <c r="M24" s="19"/>
-      <c r="N24" s="46"/>
+      <c r="N24" s="66"/>
       <c r="O24" s="19"/>
       <c r="P24" s="19"/>
       <c r="Q24" s="19"/>
       <c r="R24" s="19"/>
-      <c r="S24" s="46"/>
+      <c r="S24" s="66"/>
       <c r="T24" s="11"/>
       <c r="U24" s="1"/>
       <c r="V24" s="1"/>
@@ -2609,32 +2756,30 @@
       <c r="X24" s="1"/>
       <c r="Y24" s="1"/>
     </row>
-    <row r="25" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="25" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A25" s="1"/>
-      <c r="B25" s="55" t="s">
-        <v>36</v>
-      </c>
-      <c r="C25" s="49"/>
-      <c r="D25" s="14" t="s">
-        <v>45</v>
+      <c r="B25" s="51"/>
+      <c r="C25" s="52"/>
+      <c r="D25" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="F25" s="59"/>
-      <c r="G25" s="62"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="73"/>
       <c r="H25" s="19"/>
       <c r="I25" s="19"/>
       <c r="J25" s="19"/>
-      <c r="K25" s="20"/>
-      <c r="L25" s="19"/>
+      <c r="K25" s="19"/>
+      <c r="L25" s="39"/>
       <c r="M25" s="19"/>
-      <c r="N25" s="46"/>
+      <c r="N25" s="66"/>
       <c r="O25" s="19"/>
       <c r="P25" s="19"/>
       <c r="Q25" s="19"/>
       <c r="R25" s="19"/>
-      <c r="S25" s="46"/>
+      <c r="S25" s="66"/>
       <c r="T25" s="11"/>
       <c r="U25" s="1"/>
       <c r="V25" s="1"/>
@@ -2642,30 +2787,26 @@
       <c r="X25" s="1"/>
       <c r="Y25" s="1"/>
     </row>
-    <row r="26" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="26" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A26" s="1"/>
-      <c r="B26" s="50"/>
-      <c r="C26" s="44"/>
-      <c r="D26" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="F26" s="60"/>
-      <c r="G26" s="57"/>
+      <c r="B26" s="51"/>
+      <c r="C26" s="52"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="76"/>
+      <c r="G26" s="73"/>
       <c r="H26" s="19"/>
       <c r="I26" s="19"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="6"/>
+      <c r="J26" s="19"/>
+      <c r="K26" s="20"/>
       <c r="L26" s="19"/>
       <c r="M26" s="19"/>
-      <c r="N26" s="46"/>
+      <c r="N26" s="66"/>
       <c r="O26" s="19"/>
       <c r="P26" s="19"/>
       <c r="Q26" s="19"/>
       <c r="R26" s="19"/>
-      <c r="S26" s="46"/>
+      <c r="S26" s="66"/>
       <c r="T26" s="11"/>
       <c r="U26" s="1"/>
       <c r="V26" s="1"/>
@@ -2673,30 +2814,25 @@
       <c r="X26" s="1"/>
       <c r="Y26" s="1"/>
     </row>
-    <row r="27" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="27" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="50"/>
-      <c r="C27" s="44"/>
-      <c r="D27" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="E27" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="F27" s="60"/>
-      <c r="G27" s="57"/>
+      <c r="B27" s="45"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="77"/>
+      <c r="G27" s="74"/>
       <c r="H27" s="19"/>
       <c r="I27" s="19"/>
-      <c r="J27" s="19"/>
       <c r="K27" s="20"/>
       <c r="L27" s="19"/>
       <c r="M27" s="19"/>
-      <c r="N27" s="46"/>
+      <c r="N27" s="66"/>
       <c r="O27" s="19"/>
       <c r="P27" s="19"/>
       <c r="Q27" s="19"/>
       <c r="R27" s="19"/>
-      <c r="S27" s="46"/>
+      <c r="S27" s="66"/>
       <c r="T27" s="11"/>
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
@@ -2704,181 +2840,204 @@
       <c r="X27" s="1"/>
       <c r="Y27" s="1"/>
     </row>
-    <row r="28" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="28" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A28" s="1"/>
-      <c r="B28" s="50"/>
+      <c r="B28" s="71" t="s">
+        <v>36</v>
+      </c>
       <c r="C28" s="44"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="60"/>
-      <c r="G28" s="57"/>
+      <c r="D28" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F28" s="75"/>
+      <c r="G28" s="78"/>
       <c r="H28" s="19"/>
       <c r="I28" s="19"/>
       <c r="J28" s="19"/>
       <c r="K28" s="20"/>
-      <c r="L28" s="19"/>
-      <c r="M28" s="19"/>
-      <c r="N28" s="46"/>
+      <c r="L28" s="39"/>
+      <c r="M28" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="N28" s="66"/>
       <c r="O28" s="19"/>
       <c r="P28" s="19"/>
       <c r="Q28" s="19"/>
       <c r="R28" s="19"/>
-      <c r="S28" s="46"/>
-      <c r="T28" s="11"/>
+      <c r="S28" s="66"/>
+      <c r="T28" s="11" t="s">
+        <v>60</v>
+      </c>
       <c r="U28" s="1"/>
       <c r="V28" s="1"/>
       <c r="W28" s="1"/>
       <c r="X28" s="1"/>
       <c r="Y28" s="1"/>
     </row>
-    <row r="29" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="29" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A29" s="1"/>
-      <c r="B29" s="50"/>
-      <c r="C29" s="44"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="60"/>
-      <c r="G29" s="57"/>
+      <c r="B29" s="51"/>
+      <c r="C29" s="52"/>
+      <c r="D29" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F29" s="76"/>
+      <c r="G29" s="73"/>
       <c r="H29" s="19"/>
       <c r="I29" s="19"/>
-      <c r="J29" s="19"/>
+      <c r="J29" s="20"/>
       <c r="K29" s="20"/>
-      <c r="L29" s="19"/>
-      <c r="M29" s="19"/>
-      <c r="N29" s="46"/>
+      <c r="L29" s="20"/>
+      <c r="M29" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="N29" s="66"/>
       <c r="O29" s="19"/>
       <c r="P29" s="19"/>
       <c r="Q29" s="19"/>
       <c r="R29" s="19"/>
-      <c r="S29" s="46"/>
-      <c r="T29" s="11"/>
+      <c r="S29" s="66"/>
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
       <c r="W29" s="1"/>
       <c r="X29" s="1"/>
       <c r="Y29" s="1"/>
     </row>
-    <row r="30" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
+    <row r="30" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A30" s="1"/>
       <c r="B30" s="51"/>
       <c r="C30" s="52"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="61"/>
-      <c r="G30" s="58"/>
+      <c r="D30" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F30" s="76"/>
+      <c r="G30" s="73"/>
       <c r="H30" s="19"/>
       <c r="I30" s="19"/>
       <c r="J30" s="19"/>
-      <c r="K30" s="37"/>
-      <c r="L30" s="19"/>
-      <c r="M30" s="19"/>
-      <c r="N30" s="65"/>
+      <c r="K30" s="20"/>
+      <c r="L30" s="20"/>
+      <c r="M30" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="N30" s="66"/>
       <c r="O30" s="19"/>
       <c r="P30" s="19"/>
       <c r="Q30" s="19"/>
       <c r="R30" s="19"/>
-      <c r="S30" s="47"/>
-      <c r="T30" s="15"/>
+      <c r="S30" s="66"/>
+      <c r="T30" s="11"/>
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
       <c r="W30" s="1"/>
       <c r="X30" s="1"/>
       <c r="Y30" s="1"/>
     </row>
-    <row r="31" spans="1:26" ht="16.5" customHeight="1">
+    <row r="31" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A31" s="1"/>
-      <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
-      <c r="K31" s="38"/>
-      <c r="L31" s="1"/>
-      <c r="M31" s="1"/>
-      <c r="N31" s="1"/>
-      <c r="O31" s="1"/>
-      <c r="P31" s="1"/>
-      <c r="Q31" s="1"/>
-      <c r="R31" s="1"/>
-      <c r="S31" s="1"/>
-      <c r="T31" s="1"/>
+      <c r="B31" s="51"/>
+      <c r="C31" s="52"/>
+      <c r="D31" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F31" s="76"/>
+      <c r="G31" s="73"/>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="20"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="19"/>
+      <c r="N31" s="66"/>
+      <c r="O31" s="19"/>
+      <c r="P31" s="19"/>
+      <c r="Q31" s="19"/>
+      <c r="R31" s="19"/>
+      <c r="S31" s="66"/>
+      <c r="T31" s="11"/>
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
       <c r="W31" s="1"/>
       <c r="X31" s="1"/>
       <c r="Y31" s="1"/>
-      <c r="Z31" s="1"/>
-    </row>
-    <row r="32" spans="1:26" ht="16.5" customHeight="1">
+    </row>
+    <row r="32" spans="1:25" ht="29.25" customHeight="1" thickBot="1">
       <c r="A32" s="1"/>
-      <c r="B32" s="1"/>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-      <c r="J32" s="1"/>
-      <c r="K32" s="1"/>
-      <c r="L32" s="1"/>
-      <c r="M32" s="1"/>
-      <c r="N32" s="1"/>
-      <c r="O32" s="1"/>
-      <c r="P32" s="1"/>
-      <c r="Q32" s="1"/>
-      <c r="R32" s="1"/>
-      <c r="S32" s="1"/>
-      <c r="T32" s="1"/>
+      <c r="B32" s="51"/>
+      <c r="C32" s="52"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="76"/>
+      <c r="G32" s="73"/>
+      <c r="H32" s="19"/>
+      <c r="I32" s="19"/>
+      <c r="J32" s="19"/>
+      <c r="K32" s="20"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="19"/>
+      <c r="N32" s="66"/>
+      <c r="O32" s="19"/>
+      <c r="P32" s="19"/>
+      <c r="Q32" s="19"/>
+      <c r="R32" s="19"/>
+      <c r="S32" s="66"/>
+      <c r="T32" s="11"/>
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
       <c r="W32" s="1"/>
       <c r="X32" s="1"/>
       <c r="Y32" s="1"/>
-      <c r="Z32" s="1"/>
-    </row>
-    <row r="33" spans="1:26" ht="16.5" customHeight="1">
+    </row>
+    <row r="33" spans="1:26" ht="29.25" customHeight="1" thickBot="1">
       <c r="A33" s="1"/>
-      <c r="B33" s="1"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
-      <c r="K33" s="1"/>
-      <c r="L33" s="1"/>
-      <c r="M33" s="1"/>
-      <c r="N33" s="1"/>
-      <c r="O33" s="1"/>
-      <c r="P33" s="1"/>
-      <c r="Q33" s="1"/>
-      <c r="R33" s="1"/>
-      <c r="S33" s="1"/>
-      <c r="T33" s="1"/>
+      <c r="B33" s="45"/>
+      <c r="C33" s="47"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="77"/>
+      <c r="G33" s="74"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="19"/>
+      <c r="J33" s="19"/>
+      <c r="K33" s="37"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="19"/>
+      <c r="N33" s="82"/>
+      <c r="O33" s="19"/>
+      <c r="P33" s="19"/>
+      <c r="Q33" s="19"/>
+      <c r="R33" s="19"/>
+      <c r="S33" s="67"/>
+      <c r="T33" s="15"/>
       <c r="U33" s="1"/>
       <c r="V33" s="1"/>
       <c r="W33" s="1"/>
       <c r="X33" s="1"/>
       <c r="Y33" s="1"/>
-      <c r="Z33" s="1"/>
     </row>
     <row r="34" spans="1:26" ht="16.5" customHeight="1">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
-      <c r="C34" s="16"/>
+      <c r="C34" s="1"/>
       <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
-      <c r="K34" s="1"/>
+      <c r="K34" s="38"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
@@ -2898,7 +3057,7 @@
     <row r="35" spans="1:26" ht="16.5" customHeight="1">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
-      <c r="C35" s="16"/>
+      <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -2982,7 +3141,7 @@
     <row r="38" spans="1:26" ht="16.5" customHeight="1">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
+      <c r="C38" s="16"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
@@ -3010,7 +3169,7 @@
     <row r="39" spans="1:26" ht="16.5" customHeight="1">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
-      <c r="C39" s="1"/>
+      <c r="C39" s="16"/>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
@@ -3038,9 +3197,9 @@
     <row r="40" spans="1:26" ht="16.5" customHeight="1">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="16"/>
-      <c r="E40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
@@ -3067,8 +3226,8 @@
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
-      <c r="D41" s="16"/>
-      <c r="E41" s="16"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
@@ -3095,8 +3254,8 @@
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
-      <c r="D42" s="16"/>
-      <c r="E42" s="16"/>
+      <c r="D42" s="1"/>
+      <c r="E42" s="1"/>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
@@ -3207,8 +3366,8 @@
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="16"/>
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
@@ -3235,8 +3394,8 @@
       <c r="A47" s="1"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
-      <c r="D47" s="1"/>
-      <c r="E47" s="1"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
@@ -3263,8 +3422,8 @@
       <c r="A48" s="1"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
@@ -8383,9 +8542,90 @@
       <c r="Y230" s="1"/>
       <c r="Z230" s="1"/>
     </row>
-    <row r="231" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="232" spans="1:26" ht="15.75" customHeight="1"/>
-    <row r="233" spans="1:26" ht="15.75" customHeight="1"/>
+    <row r="231" spans="1:26" ht="16.5" customHeight="1">
+      <c r="A231" s="1"/>
+      <c r="B231" s="1"/>
+      <c r="C231" s="1"/>
+      <c r="D231" s="1"/>
+      <c r="E231" s="1"/>
+      <c r="F231" s="1"/>
+      <c r="G231" s="1"/>
+      <c r="H231" s="1"/>
+      <c r="I231" s="1"/>
+      <c r="J231" s="1"/>
+      <c r="K231" s="1"/>
+      <c r="L231" s="1"/>
+      <c r="M231" s="1"/>
+      <c r="N231" s="1"/>
+      <c r="O231" s="1"/>
+      <c r="P231" s="1"/>
+      <c r="Q231" s="1"/>
+      <c r="R231" s="1"/>
+      <c r="S231" s="1"/>
+      <c r="T231" s="1"/>
+      <c r="U231" s="1"/>
+      <c r="V231" s="1"/>
+      <c r="W231" s="1"/>
+      <c r="X231" s="1"/>
+      <c r="Y231" s="1"/>
+      <c r="Z231" s="1"/>
+    </row>
+    <row r="232" spans="1:26" ht="16.5" customHeight="1">
+      <c r="A232" s="1"/>
+      <c r="B232" s="1"/>
+      <c r="C232" s="1"/>
+      <c r="D232" s="1"/>
+      <c r="E232" s="1"/>
+      <c r="F232" s="1"/>
+      <c r="G232" s="1"/>
+      <c r="H232" s="1"/>
+      <c r="I232" s="1"/>
+      <c r="J232" s="1"/>
+      <c r="K232" s="1"/>
+      <c r="L232" s="1"/>
+      <c r="M232" s="1"/>
+      <c r="N232" s="1"/>
+      <c r="O232" s="1"/>
+      <c r="P232" s="1"/>
+      <c r="Q232" s="1"/>
+      <c r="R232" s="1"/>
+      <c r="S232" s="1"/>
+      <c r="T232" s="1"/>
+      <c r="U232" s="1"/>
+      <c r="V232" s="1"/>
+      <c r="W232" s="1"/>
+      <c r="X232" s="1"/>
+      <c r="Y232" s="1"/>
+      <c r="Z232" s="1"/>
+    </row>
+    <row r="233" spans="1:26" ht="16.5" customHeight="1">
+      <c r="A233" s="1"/>
+      <c r="B233" s="1"/>
+      <c r="C233" s="1"/>
+      <c r="D233" s="1"/>
+      <c r="E233" s="1"/>
+      <c r="F233" s="1"/>
+      <c r="G233" s="1"/>
+      <c r="H233" s="1"/>
+      <c r="I233" s="1"/>
+      <c r="J233" s="1"/>
+      <c r="K233" s="1"/>
+      <c r="L233" s="1"/>
+      <c r="M233" s="1"/>
+      <c r="N233" s="1"/>
+      <c r="O233" s="1"/>
+      <c r="P233" s="1"/>
+      <c r="Q233" s="1"/>
+      <c r="R233" s="1"/>
+      <c r="S233" s="1"/>
+      <c r="T233" s="1"/>
+      <c r="U233" s="1"/>
+      <c r="V233" s="1"/>
+      <c r="W233" s="1"/>
+      <c r="X233" s="1"/>
+      <c r="Y233" s="1"/>
+      <c r="Z233" s="1"/>
+    </row>
     <row r="234" spans="1:26" ht="15.75" customHeight="1"/>
     <row r="235" spans="1:26" ht="15.75" customHeight="1"/>
     <row r="236" spans="1:26" ht="15.75" customHeight="1"/>
@@ -9149,8 +9389,27 @@
     <row r="994" ht="15.75" customHeight="1"/>
     <row r="995" ht="15.75" customHeight="1"/>
     <row r="996" ht="15.75" customHeight="1"/>
+    <row r="997" ht="15.75" customHeight="1"/>
+    <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="T5:T7"/>
+    <mergeCell ref="S8:S33"/>
+    <mergeCell ref="B8:C16"/>
+    <mergeCell ref="B17:C21"/>
+    <mergeCell ref="B22:C27"/>
+    <mergeCell ref="B28:C33"/>
+    <mergeCell ref="G8:G16"/>
+    <mergeCell ref="F22:F27"/>
+    <mergeCell ref="G22:G27"/>
+    <mergeCell ref="F28:F33"/>
+    <mergeCell ref="G28:G33"/>
+    <mergeCell ref="F8:F16"/>
+    <mergeCell ref="N8:N33"/>
+    <mergeCell ref="F17:F21"/>
+    <mergeCell ref="H5:L5"/>
+    <mergeCell ref="G17:G21"/>
     <mergeCell ref="B2:S3"/>
     <mergeCell ref="B4:S4"/>
     <mergeCell ref="B5:C7"/>
@@ -9158,22 +9417,6 @@
     <mergeCell ref="E5:E7"/>
     <mergeCell ref="Q5:S5"/>
     <mergeCell ref="M5:P5"/>
-    <mergeCell ref="T5:T7"/>
-    <mergeCell ref="S8:S30"/>
-    <mergeCell ref="B8:C13"/>
-    <mergeCell ref="B14:C18"/>
-    <mergeCell ref="B19:C24"/>
-    <mergeCell ref="B25:C30"/>
-    <mergeCell ref="G8:G13"/>
-    <mergeCell ref="F19:F24"/>
-    <mergeCell ref="G19:G24"/>
-    <mergeCell ref="F25:F30"/>
-    <mergeCell ref="G25:G30"/>
-    <mergeCell ref="F8:F13"/>
-    <mergeCell ref="N8:N30"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="H5:L5"/>
-    <mergeCell ref="G14:G18"/>
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>